<commit_message>
herramientas-mx: loseta ligera con ventanas de 16 mm (C6: 704 a 579 g) y caso de negocio recalculado con el factor nuevo (#338)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TeXFoDoFpVre8AKoL589gf
</commit_message>
<xml_diff>
--- a/docs/herramientas-mx/caso_negocio.xlsx
+++ b/docs/herramientas-mx/caso_negocio.xlsx
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>27184.98</v>
+        <v>26254.73</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -528,7 +528,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>77187.99000000001</v>
+        <v>76257.74000000001</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>323209.18</v>
+        <v>316929.73</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>22.1</v>
+        <v>21.7</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>8.800000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -619,7 +619,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>La reposicion registrada en Odoo NO paga el plan completo en un plazo razonable (8.8 a 33.1 anios). El piloto se recupera en 0.7 a 2.8 anios y sus contenedores sirven al plan completo. El caso del plan completo depende del conteo fisico (cuanto falta de verdad) y de lo que hoy no esta medido (horas buscando herramienta, kits olvidados, compras fuera de Odoo). El piloto existe para medir eso.</t>
+          <t>La reposicion registrada en Odoo NO paga el plan completo en un plazo razonable (8.6 a 32.5 anios). El piloto se recupera en 0.7 a 2.7 anios y sus contenedores sirven al plan completo. El caso del plan completo depende del conteo fisico (cuanto falta de verdad) y de lo que hoy no esta medido (horas buscando herramienta, kits olvidados, compras fuera de Odoo). El piloto existe para medir eso.</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
@@ -2058,7 +2058,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>27184.98</v>
+        <v>26254.73</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -2075,7 +2075,7 @@
         <v>9757.01</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="3">
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>27184.98</v>
+        <v>26254.73</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -2102,7 +2102,7 @@
         <v>14635.51</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="4">
@@ -2112,7 +2112,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>27184.98</v>
+        <v>26254.73</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -2139,7 +2139,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>27184.98</v>
+        <v>26254.73</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -2166,7 +2166,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>27184.98</v>
+        <v>26254.73</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -2193,7 +2193,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>27184.98</v>
+        <v>26254.73</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -2220,7 +2220,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>323209.18</v>
+        <v>316929.73</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -2237,7 +2237,7 @@
         <v>9757.01</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>33.1</v>
+        <v>32.5</v>
       </c>
     </row>
     <row r="9">
@@ -2247,7 +2247,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>323209.18</v>
+        <v>316929.73</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -2264,7 +2264,7 @@
         <v>14635.51</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>22.1</v>
+        <v>21.7</v>
       </c>
     </row>
     <row r="10">
@@ -2274,7 +2274,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>323209.18</v>
+        <v>316929.73</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -2291,7 +2291,7 @@
         <v>17562.62</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>18.4</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11">
@@ -2301,7 +2301,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>323209.18</v>
+        <v>316929.73</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
@@ -2318,7 +2318,7 @@
         <v>20436.4</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>15.8</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="12">
@@ -2328,7 +2328,7 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>323209.18</v>
+        <v>316929.73</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
@@ -2345,7 +2345,7 @@
         <v>30654.6</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>10.5</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="13">
@@ -2355,7 +2355,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>323209.18</v>
+        <v>316929.73</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
@@ -2372,7 +2372,7 @@
         <v>36785.52</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>8.800000000000001</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="14">
@@ -2544,7 +2544,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>176863.18</v>
+        <v>170583.73</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
@@ -2561,7 +2561,7 @@
         <v>9757.01</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>18.1</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="21">
@@ -2571,7 +2571,7 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>176863.18</v>
+        <v>170583.73</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         <v>14635.51</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>12.1</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="22">
@@ -2598,7 +2598,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>176863.18</v>
+        <v>170583.73</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
         <v>17562.62</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>10.1</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="23">
@@ -2625,7 +2625,7 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>176863.18</v>
+        <v>170583.73</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
@@ -2642,7 +2642,7 @@
         <v>20436.4</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>8.699999999999999</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="24">
@@ -2652,7 +2652,7 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>176863.18</v>
+        <v>170583.73</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
@@ -2669,7 +2669,7 @@
         <v>30654.6</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="25">
@@ -2679,7 +2679,7 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>176863.18</v>
+        <v>170583.73</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
@@ -2696,7 +2696,7 @@
         <v>36785.52</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>4.8</v>
+        <v>4.6</v>
       </c>
     </row>
   </sheetData>
@@ -2813,10 +2813,10 @@
         <v>4662.75</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>37804.81</v>
+        <v>32291.98</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>273300.67</v>
+        <v>267787.84</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>5</v>
@@ -2825,10 +2825,10 @@
         <v>25</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>59.72</v>
+        <v>51.01</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>3006</v>
+        <v>2574.6</v>
       </c>
     </row>
     <row r="3">
@@ -2855,10 +2855,10 @@
         <v>7936.4</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>58347.03</v>
+        <v>49405.57</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>484791.94</v>
+        <v>475850.48</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>6</v>
@@ -2867,10 +2867,10 @@
         <v>44</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>92.18000000000001</v>
+        <v>78.05</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>4639.6</v>
+        <v>3940</v>
       </c>
     </row>
     <row r="4">
@@ -2897,10 +2897,10 @@
         <v>5357.3</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>43591.78</v>
+        <v>37312.33</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>323209.18</v>
+        <v>316929.73</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>5</v>
@@ -2909,10 +2909,10 @@
         <v>28</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>68.87</v>
+        <v>58.95</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>3466.1</v>
+        <v>2974.7</v>
       </c>
     </row>
     <row r="5">
@@ -2939,10 +2939,10 @@
         <v>9920.5</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>72933.78999999999</v>
+        <v>61756.96</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>625214.12</v>
+        <v>614037.29</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>6</v>
@@ -2951,10 +2951,10 @@
         <v>55</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>115.22</v>
+        <v>97.56</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>5799.5</v>
+        <v>4925</v>
       </c>
     </row>
     <row r="6">
@@ -2981,10 +2981,10 @@
         <v>6051.85</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>49378.76</v>
+        <v>42332.68</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>373117.7</v>
+        <v>366071.62</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>5</v>
@@ -2993,10 +2993,10 @@
         <v>31</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>78.01000000000001</v>
+        <v>66.88</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>3926.3</v>
+        <v>3374.9</v>
       </c>
     </row>
     <row r="7">
@@ -3023,10 +3023,10 @@
         <v>11904.6</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>87520.55</v>
+        <v>74108.36</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>765636.3</v>
+        <v>752224.11</v>
       </c>
       <c r="I7" s="2" t="n">
         <v>6</v>
@@ -3035,10 +3035,10 @@
         <v>66</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>138.26</v>
+        <v>117.07</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>6959.4</v>
+        <v>5910</v>
       </c>
     </row>
   </sheetData>
@@ -3140,18 +3140,18 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>PETG 10.69 kg (incluye 15 % merma)</t>
+          <t>PETG 9.22 kg (incluye 15 % merma)</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>6767.31</v>
+        <v>5837.06</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>6767.31</v>
+        <v>5837.06</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>gramos de Fase 6 x 2.28 (C6 medido 695 g contra 305 g estimados) + bandeja 8420 1640 g; 633.0/kg</t>
+          <t>gramos de Fase 6 x 1.90 (C6 medido 579 g contra 305 g estimados) + bandeja 8420 1640 g; 633.0/kg</t>
         </is>
       </c>
     </row>
@@ -3162,14 +3162,14 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>538.1</v>
+        <v>465.2</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>538.1</v>
+        <v>465.2</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Fase 6 x 2.51 (C6 medido 40.2 h contra 16.0 h) + bandeja 94.6 h. A 20 h por dia son 27 dias de impresora estandar</t>
+          <t>Fase 6 x 2.10 (C6 medido 33.6 h contra 16.0 h) + bandeja 94.6 h. A 20 h por dia son 23 dias de impresora estandar</t>
         </is>
       </c>
     </row>
@@ -3208,10 +3208,10 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>27184.98</v>
+        <v>26254.73</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>77187.99000000001</v>
+        <v>76257.74000000001</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -3895,7 +3895,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>PETG corregido por el cajon C6 medido (factor 2.28 en gramos, 2.51 en horas)</t>
+          <t>PETG corregido por el cajon C6 medido (factor 1.90 en gramos, 2.10 en horas)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
herramientas-mx: caso de negocio v2 con menudeo Jeeves, horas perdidas parametricas y recuperacion por cobertura (#338)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TeXFoDoFpVre8AKoL589gf
</commit_message>
<xml_diff>
--- a/docs/herramientas-mx/caso_negocio.xlsx
+++ b/docs/herramientas-mx/caso_negocio.xlsx
@@ -16,6 +16,11 @@
     <sheet name="Piloto_costo" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Kits_huerfanos" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Supuestos" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Jeeves_menudeo" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Jeeves_escenarios" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Horas_perdidas" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Recuperacion_v2" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Dato_vs_supuesto" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -636,6 +641,1306 @@
       <c r="C13" s="2" t="inlineStr">
         <is>
           <t>proyectos In Progress con asistencia previa y ninguna en los ultimos 10 dias habiles. Hoja Kits_huerfanos</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CASO V2 (sesion nocturna 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Menudeo Jeeves anualizado, E1 / E2 / E3</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>3,938 / 277,711 / 551,484</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>hojas Jeeves_menudeo y Jeeves_escenarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Horas perdidas en MXN al anio, bajo / medio / alto</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>24,310 / 72,920 / 145,830</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>costo hora de 100 es PARAMETRO de referencia; hoja Horas_perdidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Recuperacion del piloto, bajo / medio sin ferreteria / medio / alto (anios)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2.04 / 0.87 / 0.25 / 0.13</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>hoja Recuperacion_v2 (ya cuenta que el piloto cubre 1 de 2.8 frentes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Recuperacion del lote de 2, bajo / medio sin ferreteria / medio / alto (anios)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>4.88 / 2.09 / 0.61 / 0.32</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>acumulado de F2 del plan maestro</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Recuperacion del plan completo, bajo / medio sin ferreteria / medio / alto (anios)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>8.85 / 3.79 / 1.1 / 0.57</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>hoja Recuperacion_v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Costo de retraso con cliente</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>cualitativo</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Ejemplo: una cuadrilla de 4 en Topo Chico espera media manana una llave que se quedo en otra planta; la actividad del cronograma se recorre y, si el contrato tiene penalizacion por atraso, aplica. No se estima monto: no hay dato.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>comercio</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>cargos</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>monto MXN (ene a sep 2026)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>anualizado</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>clase</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>por que esa clase</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Ferreterias locales</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>208</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>189733.44</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>260348.52</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>incierto</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>ferreteria o tienda general: el concepto no dice que se compro</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>133761.93</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>183545.51</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>incierto</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>ferreteria o tienda general: el concepto no dice que se compro</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Mercado Libre / MercadoPago</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>51491.28</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>70655.33</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>incierto</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>ferreteria o tienda general: el concepto no dice que se compro</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Plomerama (plomeria)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>19114.47</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>26228.5</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>material_probable</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>comercio de plomeria o tornilleria: material de proyecto</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Tornillos (tornilleria)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>14522.82</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>19927.93</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>material_probable</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>comercio de plomeria o tornilleria: material de proyecto</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>14221.87</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>19514.97</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>incierto</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>ferreteria o tienda general: el concepto no dice que se compro</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Sodimac</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>5999</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>8231.709999999999</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>incierto</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>ferreteria o tienda general: el concepto no dice que se compro</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Sin comercio visible (concepto truncado)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>3825.68</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>5249.52</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>incierto</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>ferreteria o tienda general: el concepto no dice que se compro</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>DeWalt (Dwmx Herramientas)</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>2869.96</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>3938.1</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>herramienta_clara</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>el comercio es una marca de herramienta</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>EXCLUIDAS: conciliadas con factura de proveedor</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>57609.55</v>
+      </c>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>excluido</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>pagan facturas de proveedor que pueden venir de ordenes de compra ya contadas en la reposicion por OC; se excluyen para no contar doble</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>escenario</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>monto ene a sep 2026</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>anualizado</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>como salio</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>E1 solo herramienta clara</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>2869.96</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>3938.1</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>clara 2,869.96 + 0incierto 399,033.20; anualizado x 1.372 (365 / 266 dias)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>E2 clara + mitad de lo incierto</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>202386.56</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>277710.88</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>clara 2,869.96 + 0.5 x incierto 399,033.20; anualizado x 1.372 (365 / 266 dias)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>E3 clara + todo lo incierto</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>401903.16</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>551483.66</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>clara 2,869.96 + 1 x incierto 399,033.20; anualizado x 1.372 (365 / 266 dias)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Material probable (no entra)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>33637.29</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>46156.43</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>plomeria y tornilleria</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>escenario</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>minutos por frente por dia (supuesto)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>personas por frente (dato)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>frentes por dia (dato)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>dias habiles al anio (supuesto)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>horas persona al anio</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>costo hora de referencia (PARAMETRO)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>MXN al anio</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>243.1</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>24310</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>medio</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>729.2</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>72920</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>alto</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>1458.3</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>145830</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>fuente de los datos</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>735 asistencias / 175 dia-proyecto</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>175 / 63 dias</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>NO sale de nomina: valor de referencia para que direccion lo ajuste</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>inversion</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>cobertura (frentes que cubre / frentes por dia)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>escenario</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>reposicion OC al anio</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Jeeves herramienta al anio</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>horas perdidas MXN al anio</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>ahorro anual (cobertura x 75 % x suma)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>anios para recuperar</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Piloto (1 base + TUB)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>26254.73</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>19514.02</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>3938.1</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>24310</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>12895.77</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>2.04</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Piloto (1 base + TUB)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>26254.73</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>medio sin ferreteria</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>34676.25</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>3938.1</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>72920</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>30114.27</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Piloto (1 base + TUB)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>26254.73</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>medio</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>34676.25</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>277710.88</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>72920</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>104032.93</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Piloto (1 base + TUB)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>26254.73</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>alto</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>40872.8</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>551483.66</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>145830</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>199310.34</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Lote de 2 (acumulado F2, 3 bases)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>125934.52</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>19514.02</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>3938.1</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>24310</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>25791.54</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>4.88</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Lote de 2 (acumulado F2, 3 bases)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>125934.52</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>medio sin ferreteria</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>34676.25</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>3938.1</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>72920</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>60228.55</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>2.09</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Lote de 2 (acumulado F2, 3 bases)</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>125934.52</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>medio</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>34676.25</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>277710.88</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>72920</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>208065.85</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>0.61</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Lote de 2 (acumulado F2, 3 bases)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>125934.52</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>alto</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>40872.8</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>551483.66</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>145830</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>398620.69</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Plan completo (5 bases)</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>316929.73</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>19514.02</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>3938.1</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>24310</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>35821.59</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>8.85</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Plan completo (5 bases)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>316929.73</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>medio sin ferreteria</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>34676.25</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>3938.1</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>72920</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>83650.75999999999</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>3.79</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Plan completo (5 bases)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>316929.73</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>medio</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>34676.25</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>277710.88</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>72920</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>288980.35</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Plan completo (5 bases)</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>316929.73</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>alto</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>40872.8</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>551483.66</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>145830</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>553639.85</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>0.57</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>componente</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>que es dato de Odoo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>que es supuesto</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Reposicion por orden de compra</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>lineas de purchase.order.line clasificadas (18 reposicion, 2 duplicadas)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>que es un piso del gasto real; el 75 % que evita el carrito</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Menudeo en tarjeta Jeeves</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>323 cargos no conciliados por 435,540.45 en 2026-01-01, 2026-09-23, por comercio</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>que parte de ferreterias, Home Depot, Mercado Libre y Amazon es herramienta (0, 50 o 100 %)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Horas perdidas buscando o esperando</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2.78 frentes por dia y 4.20 personas por frente (kiosko, jul a sep 2026)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>minutos por dia (5, 15, 30), 250 dias habiles y el costo hora de 100 (parametro, no nomina)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Costo de retraso con cliente</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>nada: no se inventa monto</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>linea cualitativa: ver Resumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Cobertura de cada inversion</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>frentes por dia (kiosko)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>que un carrito cubre un frente; el lote de 2 cubre 2 frentes activos y 1 de reserva</t>
         </is>
       </c>
     </row>

</xml_diff>